<commit_message>
Cập nhật screener_cache.xlsx 2026-10-09 22:30
</commit_message>
<xml_diff>
--- a/screener_cache.xlsx
+++ b/screener_cache.xlsx
@@ -535,19 +535,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20.15</v>
+        <v>20.1</v>
       </c>
       <c r="C2" t="n">
-        <v>257.89</v>
+        <v>328.71</v>
       </c>
       <c r="D2" t="n">
-        <v>12798551</v>
+        <v>16353579</v>
       </c>
       <c r="E2" t="n">
-        <v>18097622</v>
+        <v>17817678</v>
       </c>
       <c r="F2" t="n">
-        <v>0.71</v>
+        <v>0.92</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -565,13 +565,13 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>21.42</v>
+        <v>21.28</v>
       </c>
       <c r="K2" t="n">
         <v>22.95</v>
       </c>
       <c r="L2" t="n">
-        <v>-12.19</v>
+        <v>-12.4</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -587,10 +587,10 @@
         </is>
       </c>
       <c r="R2" t="n">
-        <v>23.08</v>
+        <v>27.27</v>
       </c>
       <c r="S2" t="n">
-        <v>18.69</v>
+        <v>18.72</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -615,19 +615,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19.05</v>
+        <v>19</v>
       </c>
       <c r="C3" t="n">
-        <v>486.96</v>
+        <v>501.37</v>
       </c>
       <c r="D3" t="n">
-        <v>25562307</v>
+        <v>26387938</v>
       </c>
       <c r="E3" t="n">
-        <v>22305650</v>
+        <v>22036361</v>
       </c>
       <c r="F3" t="n">
-        <v>1.15</v>
+        <v>1.2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
         <v>20.17</v>
       </c>
       <c r="L3" t="n">
-        <v>-5.55</v>
+        <v>-5.8</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>7.27</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>16.34</v>
+        <v>17.39</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -684,7 +684,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -695,23 +695,23 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13.1</v>
+        <v>13.2</v>
       </c>
       <c r="C4" t="n">
-        <v>170.79</v>
+        <v>232.53</v>
       </c>
       <c r="D4" t="n">
-        <v>13037635</v>
+        <v>17615912</v>
       </c>
       <c r="E4" t="n">
-        <v>10451811</v>
+        <v>10534650</v>
       </c>
       <c r="F4" t="n">
-        <v>1.25</v>
+        <v>1.67</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>⚡ Có Tín Hiệu</t>
+          <t>🔥 Tiền Vào Mạnh</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -725,13 +725,13 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>15.75</v>
+        <v>15.25</v>
       </c>
       <c r="K4" t="n">
-        <v>16.08</v>
+        <v>15.85</v>
       </c>
       <c r="L4" t="n">
-        <v>-18.51</v>
+        <v>-16.72</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="R4" t="n">
-        <v>21.62</v>
+        <v>27.27</v>
       </c>
       <c r="S4" t="n">
-        <v>15.83</v>
+        <v>15.5</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -775,23 +775,23 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>59.7</v>
+        <v>57.9</v>
       </c>
       <c r="C5" t="n">
-        <v>445.79</v>
+        <v>707.9400000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>7467170</v>
+        <v>12226887</v>
       </c>
       <c r="E5" t="n">
-        <v>5090596</v>
+        <v>5346285</v>
       </c>
       <c r="F5" t="n">
-        <v>1.47</v>
+        <v>2.29</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>⚡ Có Tín Hiệu</t>
+          <t>🔥 Tiền Vào Mạnh</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -811,7 +811,7 @@
         <v>63.27</v>
       </c>
       <c r="L5" t="n">
-        <v>-5.65</v>
+        <v>-8.49</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>15.38</v>
+        <v>12.54</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -844,7 +844,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -855,23 +855,23 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31.9</v>
+        <v>32.35</v>
       </c>
       <c r="C6" t="n">
-        <v>862.96</v>
+        <v>492.89</v>
       </c>
       <c r="D6" t="n">
-        <v>27052176</v>
+        <v>15236087</v>
       </c>
       <c r="E6" t="n">
-        <v>17168583</v>
+        <v>16475504</v>
       </c>
       <c r="F6" t="n">
-        <v>1.58</v>
+        <v>0.92</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>🔥 Tiền Vào Mạnh</t>
+          <t>💤 Tiền Yếu</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -891,7 +891,7 @@
         <v>31.5</v>
       </c>
       <c r="L6" t="n">
-        <v>1.27</v>
+        <v>2.7</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -911,10 +911,10 @@
         </is>
       </c>
       <c r="R6" t="n">
-        <v>53.12</v>
+        <v>51.09</v>
       </c>
       <c r="S6" t="n">
-        <v>53.83</v>
+        <v>62.42</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -939,23 +939,23 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18.9</v>
+        <v>19.05</v>
       </c>
       <c r="C7" t="n">
-        <v>211.57</v>
+        <v>269.47</v>
       </c>
       <c r="D7" t="n">
-        <v>11194407</v>
+        <v>14145209</v>
       </c>
       <c r="E7" t="n">
-        <v>11766385</v>
+        <v>11552185</v>
       </c>
       <c r="F7" t="n">
-        <v>0.95</v>
+        <v>1.22</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>💤 Tiền Yếu</t>
+          <t>⚡ Có Tín Hiệu</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>20.15</v>
+        <v>20</v>
       </c>
       <c r="K7" t="n">
         <v>20.57</v>
       </c>
       <c r="L7" t="n">
-        <v>-8.119999999999999</v>
+        <v>-7.39</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -991,10 +991,10 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>25</v>
+        <v>18.92</v>
       </c>
       <c r="S7" t="n">
-        <v>17.4</v>
+        <v>17.48</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -1019,19 +1019,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>76.09999999999999</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>496.58</v>
+        <v>389.14</v>
       </c>
       <c r="D8" t="n">
-        <v>6525324</v>
+        <v>5126949</v>
       </c>
       <c r="E8" t="n">
-        <v>3107216</v>
+        <v>3085422</v>
       </c>
       <c r="F8" t="n">
-        <v>2.1</v>
+        <v>1.66</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
         <v>73.36</v>
       </c>
       <c r="L8" t="n">
-        <v>3.73</v>
+        <v>3.46</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1071,10 +1071,10 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>70.18000000000001</v>
+        <v>74.04000000000001</v>
       </c>
       <c r="S8" t="n">
-        <v>83.58</v>
+        <v>76.89</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>228</v>
+        <v>225.5</v>
       </c>
       <c r="C9" t="n">
-        <v>768.92</v>
+        <v>686.14</v>
       </c>
       <c r="D9" t="n">
-        <v>3372436</v>
+        <v>3042771</v>
       </c>
       <c r="E9" t="n">
-        <v>3536881</v>
+        <v>3472303</v>
       </c>
       <c r="F9" t="n">
-        <v>0.95</v>
+        <v>0.88</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1132,10 +1132,10 @@
         <v>229.8</v>
       </c>
       <c r="K9" t="n">
-        <v>207.15</v>
+        <v>213.45</v>
       </c>
       <c r="L9" t="n">
-        <v>10.07</v>
+        <v>5.65</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1151,10 +1151,10 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>38.78</v>
+        <v>41.38</v>
       </c>
       <c r="S9" t="n">
-        <v>43.31</v>
+        <v>44.16</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -1179,23 +1179,23 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>65.7</v>
+        <v>66</v>
       </c>
       <c r="C10" t="n">
-        <v>767.28</v>
+        <v>553.88</v>
       </c>
       <c r="D10" t="n">
-        <v>11678545</v>
+        <v>8392151</v>
       </c>
       <c r="E10" t="n">
-        <v>9179922</v>
+        <v>9208847</v>
       </c>
       <c r="F10" t="n">
-        <v>1.27</v>
+        <v>0.91</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>⚡ Có Tín Hiệu</t>
+          <t>💤 Tiền Yếu</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1212,17 +1212,21 @@
         <v>71.40000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>70.18000000000001</v>
+        <v>71.31</v>
       </c>
       <c r="L10" t="n">
-        <v>-6.38</v>
+        <v>-7.44</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>📉 Rẻ (dưới/sát 129)</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
@@ -1231,10 +1235,10 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>35.98</v>
+        <v>43.56</v>
       </c>
       <c r="S10" t="n">
-        <v>42.52</v>
+        <v>46.41</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1248,7 +1252,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>
@@ -1259,19 +1263,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>57.9</v>
+        <v>57.7</v>
       </c>
       <c r="C11" t="n">
-        <v>102.41</v>
+        <v>78.45</v>
       </c>
       <c r="D11" t="n">
-        <v>1768758</v>
+        <v>1359671</v>
       </c>
       <c r="E11" t="n">
-        <v>2458982</v>
+        <v>2324558</v>
       </c>
       <c r="F11" t="n">
-        <v>0.72</v>
+        <v>0.58</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1295,7 +1299,7 @@
         <v>59.5</v>
       </c>
       <c r="L11" t="n">
-        <v>-2.69</v>
+        <v>-3.03</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1311,10 +1315,10 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>31.03</v>
+        <v>33.75</v>
       </c>
       <c r="S11" t="n">
-        <v>26.48</v>
+        <v>27.61</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -1328,7 +1332,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-10-08 22:48:20</t>
+          <t>2026-10-09 22:30:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cập nhật screener_cache.xlsx 2026-10-13 23:16
</commit_message>
<xml_diff>
--- a/screener_cache.xlsx
+++ b/screener_cache.xlsx
@@ -535,19 +535,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20.1</v>
+        <v>20.45</v>
       </c>
       <c r="C2" t="n">
-        <v>328.71</v>
+        <v>243.4</v>
       </c>
       <c r="D2" t="n">
-        <v>16353579</v>
+        <v>11902095</v>
       </c>
       <c r="E2" t="n">
-        <v>17817678</v>
+        <v>17181794</v>
       </c>
       <c r="F2" t="n">
-        <v>0.92</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -565,13 +565,13 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>21.28</v>
+        <v>21.12</v>
       </c>
       <c r="K2" t="n">
         <v>22.95</v>
       </c>
       <c r="L2" t="n">
-        <v>-12.4</v>
+        <v>-10.88</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -587,10 +587,10 @@
         </is>
       </c>
       <c r="R2" t="n">
-        <v>27.27</v>
+        <v>36</v>
       </c>
       <c r="S2" t="n">
-        <v>18.72</v>
+        <v>23.34</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -615,23 +615,23 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="C3" t="n">
-        <v>501.37</v>
+        <v>288.69</v>
       </c>
       <c r="D3" t="n">
-        <v>26387938</v>
+        <v>15274729</v>
       </c>
       <c r="E3" t="n">
-        <v>22036361</v>
+        <v>21557461</v>
       </c>
       <c r="F3" t="n">
-        <v>1.2</v>
+        <v>0.71</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>⚡ Có Tín Hiệu</t>
+          <t>💤 Tiền Yếu</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -651,7 +651,7 @@
         <v>20.17</v>
       </c>
       <c r="L3" t="n">
-        <v>-5.8</v>
+        <v>-6.29</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>8.699999999999999</v>
+        <v>6.38</v>
       </c>
       <c r="S3" t="n">
-        <v>17.39</v>
+        <v>17.3</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -684,7 +684,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -695,23 +695,23 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13.2</v>
+        <v>12.9</v>
       </c>
       <c r="C4" t="n">
-        <v>232.53</v>
+        <v>138.47</v>
       </c>
       <c r="D4" t="n">
-        <v>17615912</v>
+        <v>10734107</v>
       </c>
       <c r="E4" t="n">
-        <v>10534650</v>
+        <v>10178855</v>
       </c>
       <c r="F4" t="n">
-        <v>1.67</v>
+        <v>1.05</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>🔥 Tiền Vào Mạnh</t>
+          <t>⚡ Có Tín Hiệu</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -725,13 +725,13 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>15.25</v>
+        <v>15.23</v>
       </c>
       <c r="K4" t="n">
         <v>15.85</v>
       </c>
       <c r="L4" t="n">
-        <v>-16.72</v>
+        <v>-18.61</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="R4" t="n">
-        <v>27.27</v>
+        <v>21.74</v>
       </c>
       <c r="S4" t="n">
-        <v>15.5</v>
+        <v>15</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -775,23 +775,23 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>57.9</v>
+        <v>56.3</v>
       </c>
       <c r="C5" t="n">
-        <v>707.9400000000001</v>
+        <v>438.98</v>
       </c>
       <c r="D5" t="n">
-        <v>12226887</v>
+        <v>7797089</v>
       </c>
       <c r="E5" t="n">
-        <v>5346285</v>
+        <v>5400064</v>
       </c>
       <c r="F5" t="n">
-        <v>2.29</v>
+        <v>1.44</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>🔥 Tiền Vào Mạnh</t>
+          <t>⚡ Có Tín Hiệu</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -811,7 +811,7 @@
         <v>63.27</v>
       </c>
       <c r="L5" t="n">
-        <v>-8.49</v>
+        <v>-11.02</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>12.54</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -844,7 +844,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -855,23 +855,23 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>32.35</v>
+        <v>32.95</v>
       </c>
       <c r="C6" t="n">
-        <v>492.89</v>
+        <v>765.09</v>
       </c>
       <c r="D6" t="n">
-        <v>15236087</v>
+        <v>23219651</v>
       </c>
       <c r="E6" t="n">
-        <v>16475504</v>
+        <v>17046217</v>
       </c>
       <c r="F6" t="n">
-        <v>0.92</v>
+        <v>1.36</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>💤 Tiền Yếu</t>
+          <t>⚡ Có Tín Hiệu</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>🌫️ Trong Mây</t>
+          <t>☁️ Trên Mây</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -891,7 +891,7 @@
         <v>31.5</v>
       </c>
       <c r="L6" t="n">
-        <v>2.7</v>
+        <v>4.6</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -911,10 +911,10 @@
         </is>
       </c>
       <c r="R6" t="n">
-        <v>51.09</v>
+        <v>56.31</v>
       </c>
       <c r="S6" t="n">
-        <v>62.42</v>
+        <v>64.15000000000001</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -942,20 +942,20 @@
         <v>19.05</v>
       </c>
       <c r="C7" t="n">
-        <v>269.47</v>
+        <v>127.09</v>
       </c>
       <c r="D7" t="n">
-        <v>14145209</v>
+        <v>6671584</v>
       </c>
       <c r="E7" t="n">
-        <v>11552185</v>
+        <v>11065949</v>
       </c>
       <c r="F7" t="n">
-        <v>1.22</v>
+        <v>0.6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>⚡ Có Tín Hiệu</t>
+          <t>💤 Tiền Yếu</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>20</v>
+        <v>19.96</v>
       </c>
       <c r="K7" t="n">
         <v>20.57</v>
@@ -991,10 +991,10 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>18.92</v>
+        <v>20</v>
       </c>
       <c r="S7" t="n">
-        <v>17.48</v>
+        <v>22.62</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -1019,19 +1019,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>75.90000000000001</v>
+        <v>74.8</v>
       </c>
       <c r="C8" t="n">
-        <v>389.14</v>
+        <v>747.4</v>
       </c>
       <c r="D8" t="n">
-        <v>5126949</v>
+        <v>9991979</v>
       </c>
       <c r="E8" t="n">
-        <v>3085422</v>
+        <v>3306418</v>
       </c>
       <c r="F8" t="n">
-        <v>1.66</v>
+        <v>3.02</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
         <v>73.36</v>
       </c>
       <c r="L8" t="n">
-        <v>3.46</v>
+        <v>1.96</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1067,18 +1067,18 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>🎯 BẮT ĐÁY (Vol 3.0x + giá chiết khấu 129)</t>
         </is>
       </c>
       <c r="R8" t="n">
-        <v>74.04000000000001</v>
+        <v>63.81</v>
       </c>
       <c r="S8" t="n">
-        <v>76.89</v>
+        <v>64.06999999999999</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>🔴 Bán (vùng quá mua)</t>
+          <t>⏸️ Chờ (giữa biên độ)</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>225.5</v>
+        <v>222</v>
       </c>
       <c r="C9" t="n">
-        <v>686.14</v>
+        <v>698.37</v>
       </c>
       <c r="D9" t="n">
-        <v>3042771</v>
+        <v>3145816</v>
       </c>
       <c r="E9" t="n">
-        <v>3472303</v>
+        <v>3421830</v>
       </c>
       <c r="F9" t="n">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1125,17 +1125,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>☁️ Trên Mây</t>
+          <t>🌧️ Dưới Mây</t>
         </is>
       </c>
       <c r="J9" t="n">
         <v>229.8</v>
       </c>
       <c r="K9" t="n">
-        <v>213.45</v>
+        <v>215.6</v>
       </c>
       <c r="L9" t="n">
-        <v>5.65</v>
+        <v>2.97</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1151,14 +1151,14 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>41.38</v>
+        <v>28.11</v>
       </c>
       <c r="S9" t="n">
-        <v>44.16</v>
+        <v>38.33</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>⏸️ Chờ (giữa biên độ)</t>
+          <t>🟢 Mua (vùng quá bán)</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -1179,19 +1179,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>66</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>553.88</v>
+        <v>345.16</v>
       </c>
       <c r="D10" t="n">
-        <v>8392151</v>
+        <v>5359692</v>
       </c>
       <c r="E10" t="n">
-        <v>9208847</v>
+        <v>8881614</v>
       </c>
       <c r="F10" t="n">
-        <v>0.91</v>
+        <v>0.6</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1209,24 +1209,20 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>71.40000000000001</v>
+        <v>70.95</v>
       </c>
       <c r="K10" t="n">
-        <v>71.31</v>
+        <v>72.78</v>
       </c>
       <c r="L10" t="n">
-        <v>-7.44</v>
+        <v>-11.51</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>📉 Rẻ (dưới/sát 129)</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
@@ -1235,10 +1231,10 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>43.56</v>
+        <v>34.94</v>
       </c>
       <c r="S10" t="n">
-        <v>46.41</v>
+        <v>48.13</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1252,7 +1248,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>
@@ -1263,19 +1259,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>57.7</v>
+        <v>58</v>
       </c>
       <c r="C11" t="n">
-        <v>78.45</v>
+        <v>96.29000000000001</v>
       </c>
       <c r="D11" t="n">
-        <v>1359671</v>
+        <v>1660137</v>
       </c>
       <c r="E11" t="n">
-        <v>2324558</v>
+        <v>2214716</v>
       </c>
       <c r="F11" t="n">
-        <v>0.58</v>
+        <v>0.75</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1299,7 +1295,7 @@
         <v>59.5</v>
       </c>
       <c r="L11" t="n">
-        <v>-3.03</v>
+        <v>-2.52</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1315,10 +1311,10 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>33.75</v>
+        <v>28.38</v>
       </c>
       <c r="S11" t="n">
-        <v>27.61</v>
+        <v>21.56</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -1332,7 +1328,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-10-09 22:30:13</t>
+          <t>2026-10-13 23:16:41</t>
         </is>
       </c>
     </row>

</xml_diff>